<commit_message>
Add subscriptions admin, riders API, driver-doc GET, Kirana PWA shell
- Subscriptions: /admins/subscriptions page + api/subscriptions routes for
  granting/revoking driver sachet plans; new subscriptions surface in rbac.
- Riders read API: GET /api/riders (search + pagination) and /api/riders/[id]
  with recent rides and lifetime stats.
- Driver document GET handler alongside existing PATCH/DELETE; requireRead
  helper added to apiAuth.
- Kirana PWA shell: manifest.webmanifest scoped to /k/, service worker
  (cache-first static, network-first kirana APIs, offline fallback),
  install prompt, 192/512/maskable/apple-touch icons generated via
  scripts/build-pwa-icons.py, Service-Worker-Allowed header in next.config.
- Spec script updated to reflect shipped state; xlsx regenerated.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Glimmora_Go_Spec.xlsx
+++ b/docs/Glimmora_Go_Spec.xlsx
@@ -178,7 +178,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -205,9 +205,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1834,7 +1831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G74"/>
+  <dimension ref="A1:G79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2632,12 +2629,12 @@
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>Document file upload</t>
+          <t>Document file upload UI</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>Actually uploading files to storage</t>
+          <t>Pick type + file, POST /api/uploads/driver-doc, stored under public/uploads/drivers/</t>
         </is>
       </c>
       <c r="E28" s="6" t="inlineStr">
@@ -2645,16 +2642,12 @@
           <t>SUPER/ADMIN/CITY/VERIF</t>
         </is>
       </c>
-      <c r="F28" s="16" t="inlineStr">
-        <is>
-          <t>TODO</t>
-        </is>
-      </c>
-      <c r="G28" s="6" t="inlineStr">
-        <is>
-          <t>fileUrl field exists but no upload UI</t>
-        </is>
-      </c>
+      <c r="F28" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="13" t="inlineStr">
@@ -2701,175 +2694,181 @@
       <c r="G30" s="6" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="13" t="inlineStr">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>Riders JSON API</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t>GET /api/riders (q/limit/offset), GET /api/riders/[id] with rides + stats</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="inlineStr">
+        <is>
+          <t>riders:read</t>
+        </is>
+      </c>
+      <c r="F31" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G31" s="6" t="inlineStr">
+        <is>
+          <t>For external clients and future rider app</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="13" t="inlineStr">
         <is>
           <t>FARES</t>
         </is>
       </c>
-      <c r="B31" s="14" t="n"/>
-      <c r="C31" s="14" t="n"/>
-      <c r="D31" s="14" t="n"/>
-      <c r="E31" s="14" t="n"/>
-      <c r="F31" s="14" t="n"/>
-      <c r="G31" s="15" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="6" t="n">
-        <v>23</v>
-      </c>
-      <c r="B32" s="6" t="inlineStr">
-        <is>
-          <t>/fares</t>
-        </is>
-      </c>
-      <c r="C32" s="6" t="inlineStr">
-        <is>
-          <t>Per-city fare editor</t>
-        </is>
-      </c>
-      <c r="D32" s="6" t="inlineStr">
-        <is>
-          <t>Base fare, per km, per min, minimum fare</t>
-        </is>
-      </c>
-      <c r="E32" s="6" t="inlineStr">
-        <is>
-          <t>SUPER/ADMIN/CITY (write) · VIEW (read)</t>
-        </is>
-      </c>
-      <c r="F32" s="12" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="G32" s="6" t="inlineStr">
-        <is>
-          <t>CITY sees own city only</t>
-        </is>
-      </c>
+      <c r="B32" s="14" t="n"/>
+      <c r="C32" s="14" t="n"/>
+      <c r="D32" s="14" t="n"/>
+      <c r="E32" s="14" t="n"/>
+      <c r="F32" s="14" t="n"/>
+      <c r="G32" s="15" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>/fares</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>Per-city fare editor</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>Base fare, per km, per min, minimum fare</t>
+        </is>
+      </c>
+      <c r="E33" s="6" t="inlineStr">
+        <is>
+          <t>SUPER/ADMIN/CITY (write) · VIEW (read)</t>
+        </is>
+      </c>
+      <c r="F33" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G33" s="6" t="inlineStr">
+        <is>
+          <t>CITY sees own city only</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="n">
         <v>24</v>
       </c>
-      <c r="B33" s="6" t="inlineStr">
+      <c r="B34" s="6" t="inlineStr">
         <is>
           <t>/fares</t>
         </is>
       </c>
-      <c r="C33" s="6" t="inlineStr">
+      <c r="C34" s="6" t="inlineStr">
         <is>
           <t>Saved ✓ feedback</t>
         </is>
       </c>
-      <c r="D33" s="6" t="inlineStr">
+      <c r="D34" s="6" t="inlineStr">
         <is>
           <t>2s confirmation after PUT</t>
         </is>
       </c>
-      <c r="E33" s="6" t="inlineStr">
+      <c r="E34" s="6" t="inlineStr">
         <is>
           <t>same</t>
         </is>
       </c>
-      <c r="F33" s="12" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="G33" s="6" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="13" t="inlineStr">
+      <c r="F34" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G34" s="6" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="13" t="inlineStr">
         <is>
           <t>CONCESSIONS</t>
         </is>
       </c>
-      <c r="B34" s="14" t="n"/>
-      <c r="C34" s="14" t="n"/>
-      <c r="D34" s="14" t="n"/>
-      <c r="E34" s="14" t="n"/>
-      <c r="F34" s="14" t="n"/>
-      <c r="G34" s="15" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="6" t="n">
+      <c r="B35" s="14" t="n"/>
+      <c r="C35" s="14" t="n"/>
+      <c r="D35" s="14" t="n"/>
+      <c r="E35" s="14" t="n"/>
+      <c r="F35" s="14" t="n"/>
+      <c r="G35" s="15" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="n">
         <v>25</v>
       </c>
-      <c r="B35" s="6" t="inlineStr">
+      <c r="B36" s="6" t="inlineStr">
         <is>
           <t>/concessions</t>
         </is>
       </c>
-      <c r="C35" s="6" t="inlineStr">
+      <c r="C36" s="6" t="inlineStr">
         <is>
           <t>Per-city multipliers</t>
         </is>
       </c>
-      <c r="D35" s="6" t="inlineStr">
+      <c r="D36" s="6" t="inlineStr">
         <is>
           <t>Women, senior, children — default 0.85/0.80/0.90</t>
         </is>
       </c>
-      <c r="E35" s="6" t="inlineStr">
+      <c r="E36" s="6" t="inlineStr">
         <is>
           <t>SUPER/ADMIN (write) · VIEW (read)</t>
         </is>
       </c>
-      <c r="F35" s="12" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="G35" s="6" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="13" t="inlineStr">
+      <c r="F36" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G36" s="6" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="13" t="inlineStr">
         <is>
           <t>COUPONS</t>
         </is>
       </c>
-      <c r="B36" s="14" t="n"/>
-      <c r="C36" s="14" t="n"/>
-      <c r="D36" s="14" t="n"/>
-      <c r="E36" s="14" t="n"/>
-      <c r="F36" s="14" t="n"/>
-      <c r="G36" s="15" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="6" t="n">
-        <v>26</v>
-      </c>
-      <c r="B37" s="6" t="inlineStr">
-        <is>
-          <t>/coupons</t>
-        </is>
-      </c>
-      <c r="C37" s="6" t="inlineStr">
-        <is>
-          <t>Create coupon</t>
-        </is>
-      </c>
-      <c r="D37" s="6" t="inlineStr">
-        <is>
-          <t>Code, description, FLAT/PERCENT, amount, usage limit, expiry</t>
-        </is>
-      </c>
-      <c r="E37" s="6" t="inlineStr">
-        <is>
-          <t>SUPER/ADMIN</t>
-        </is>
-      </c>
-      <c r="F37" s="12" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="G37" s="6" t="inlineStr"/>
+      <c r="B37" s="14" t="n"/>
+      <c r="C37" s="14" t="n"/>
+      <c r="D37" s="14" t="n"/>
+      <c r="E37" s="14" t="n"/>
+      <c r="F37" s="14" t="n"/>
+      <c r="G37" s="15" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="6" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
@@ -2878,17 +2877,17 @@
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>List + usage stats</t>
+          <t>Create coupon</t>
         </is>
       </c>
       <c r="D38" s="6" t="inlineStr">
         <is>
-          <t>Used count / limit, expiry date, active/disabled/expired badge</t>
+          <t>Code, description, FLAT/PERCENT, amount, usage limit, expiry</t>
         </is>
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>same + VIEW read</t>
+          <t>SUPER/ADMIN</t>
         </is>
       </c>
       <c r="F38" s="12" t="inlineStr">
@@ -2900,86 +2899,82 @@
     </row>
     <row r="39">
       <c r="A39" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>/coupons</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>List + usage stats</t>
+        </is>
+      </c>
+      <c r="D39" s="6" t="inlineStr">
+        <is>
+          <t>Used count / limit, expiry date, active/disabled/expired badge</t>
+        </is>
+      </c>
+      <c r="E39" s="6" t="inlineStr">
+        <is>
+          <t>same + VIEW read</t>
+        </is>
+      </c>
+      <c r="F39" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G39" s="6" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="n">
         <v>28</v>
       </c>
-      <c r="B39" s="6" t="inlineStr">
+      <c r="B40" s="6" t="inlineStr">
         <is>
           <t>/coupons</t>
         </is>
       </c>
-      <c r="C39" s="6" t="inlineStr">
+      <c r="C40" s="6" t="inlineStr">
         <is>
           <t>Disable / Enable / Delete</t>
         </is>
       </c>
-      <c r="D39" s="6" t="inlineStr">
+      <c r="D40" s="6" t="inlineStr">
         <is>
           <t>PATCH active flag / DELETE</t>
         </is>
       </c>
-      <c r="E39" s="6" t="inlineStr">
+      <c r="E40" s="6" t="inlineStr">
         <is>
           <t>SUPER/ADMIN</t>
         </is>
       </c>
-      <c r="F39" s="12" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="G39" s="6" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="13" t="inlineStr">
+      <c r="F40" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G40" s="6" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="13" t="inlineStr">
         <is>
           <t>CITIES</t>
         </is>
       </c>
-      <c r="B40" s="14" t="n"/>
-      <c r="C40" s="14" t="n"/>
-      <c r="D40" s="14" t="n"/>
-      <c r="E40" s="14" t="n"/>
-      <c r="F40" s="14" t="n"/>
-      <c r="G40" s="15" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="6" t="n">
-        <v>29</v>
-      </c>
-      <c r="B41" s="6" t="inlineStr">
-        <is>
-          <t>/cities</t>
-        </is>
-      </c>
-      <c r="C41" s="6" t="inlineStr">
-        <is>
-          <t>Archetype defaults editor</t>
-        </is>
-      </c>
-      <c r="D41" s="6" t="inlineStr">
-        <is>
-          <t>Per-archetype (Metro/Small Town) defaults: radius, surge, payment options, base, perKm, perMin, minFare</t>
-        </is>
-      </c>
-      <c r="E41" s="6" t="inlineStr">
-        <is>
-          <t>SUPER/ADMIN (write) · VIEW (read)</t>
-        </is>
-      </c>
-      <c r="F41" s="12" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="G41" s="6" t="inlineStr">
-        <is>
-          <t>New cities inherit these</t>
-        </is>
-      </c>
+      <c r="B41" s="14" t="n"/>
+      <c r="C41" s="14" t="n"/>
+      <c r="D41" s="14" t="n"/>
+      <c r="E41" s="14" t="n"/>
+      <c r="F41" s="14" t="n"/>
+      <c r="G41" s="15" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="6" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
@@ -2988,17 +2983,17 @@
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>Add city form</t>
+          <t>Archetype defaults editor</t>
         </is>
       </c>
       <c r="D42" s="6" t="inlineStr">
         <is>
-          <t>Name + state + archetype</t>
+          <t>Per-archetype (Metro/Small Town) defaults: radius, surge, payment options, base, perKm, perMin, minFare</t>
         </is>
       </c>
       <c r="E42" s="6" t="inlineStr">
         <is>
-          <t>SUPER/ADMIN</t>
+          <t>SUPER/ADMIN (write) · VIEW (read)</t>
         </is>
       </c>
       <c r="F42" s="12" t="inlineStr">
@@ -3006,86 +3001,90 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G42" s="6" t="inlineStr"/>
+      <c r="G42" s="6" t="inlineStr">
+        <is>
+          <t>New cities inherit these</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>/cities</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>Add city form</t>
+        </is>
+      </c>
+      <c r="D43" s="6" t="inlineStr">
+        <is>
+          <t>Name + state + archetype</t>
+        </is>
+      </c>
+      <c r="E43" s="6" t="inlineStr">
+        <is>
+          <t>SUPER/ADMIN</t>
+        </is>
+      </c>
+      <c r="F43" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G43" s="6" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="n">
         <v>31</v>
       </c>
-      <c r="B43" s="6" t="inlineStr">
+      <c r="B44" s="6" t="inlineStr">
         <is>
           <t>/cities</t>
         </is>
       </c>
-      <c r="C43" s="6" t="inlineStr">
+      <c r="C44" s="6" t="inlineStr">
         <is>
           <t>Per-city edit row</t>
         </is>
       </c>
-      <c r="D43" s="6" t="inlineStr">
+      <c r="D44" s="6" t="inlineStr">
         <is>
           <t>Archetype override, matching radius, surge, active toggle, payment pills</t>
         </is>
       </c>
-      <c r="E43" s="6" t="inlineStr">
+      <c r="E44" s="6" t="inlineStr">
         <is>
           <t>SUPER/ADMIN</t>
         </is>
       </c>
-      <c r="F43" s="12" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="G43" s="6" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="13" t="inlineStr">
+      <c r="F44" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G44" s="6" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="13" t="inlineStr">
         <is>
           <t>REFERRALS</t>
         </is>
       </c>
-      <c r="B44" s="14" t="n"/>
-      <c r="C44" s="14" t="n"/>
-      <c r="D44" s="14" t="n"/>
-      <c r="E44" s="14" t="n"/>
-      <c r="F44" s="14" t="n"/>
-      <c r="G44" s="15" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="6" t="n">
-        <v>32</v>
-      </c>
-      <c r="B45" s="6" t="inlineStr">
-        <is>
-          <t>/referrals</t>
-        </is>
-      </c>
-      <c r="C45" s="6" t="inlineStr">
-        <is>
-          <t>Stat cards</t>
-        </is>
-      </c>
-      <c r="D45" s="6" t="inlineStr">
-        <is>
-          <t>Total / joined / rewarded with conversion %</t>
-        </is>
-      </c>
-      <c r="E45" s="6" t="inlineStr">
-        <is>
-          <t>SUPER/ADMIN (write) · VIEW (read)</t>
-        </is>
-      </c>
-      <c r="F45" s="12" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="G45" s="6" t="inlineStr"/>
+      <c r="B45" s="14" t="n"/>
+      <c r="C45" s="14" t="n"/>
+      <c r="D45" s="14" t="n"/>
+      <c r="E45" s="14" t="n"/>
+      <c r="F45" s="14" t="n"/>
+      <c r="G45" s="15" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="6" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
@@ -3094,17 +3093,17 @@
       </c>
       <c r="C46" s="6" t="inlineStr">
         <is>
-          <t>Top referrers list</t>
+          <t>Stat cards</t>
         </is>
       </c>
       <c r="D46" s="6" t="inlineStr">
         <is>
-          <t>Top 5 drivers by referredDrivers count</t>
+          <t>Total / joined / rewarded with conversion %</t>
         </is>
       </c>
       <c r="E46" s="6" t="inlineStr">
         <is>
-          <t>same</t>
+          <t>SUPER/ADMIN (write) · VIEW (read)</t>
         </is>
       </c>
       <c r="F46" s="12" t="inlineStr">
@@ -3116,7 +3115,7 @@
     </row>
     <row r="47">
       <c r="A47" s="6" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
@@ -3125,12 +3124,12 @@
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>Recent referrals table</t>
+          <t>Top referrers list</t>
         </is>
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
-          <t>Referee phone, rides done / 10, status (Pending/Joined/Rewarded), date</t>
+          <t>Top 5 drivers by referredDrivers count</t>
         </is>
       </c>
       <c r="E47" s="6" t="inlineStr">
@@ -3147,7 +3146,7 @@
     </row>
     <row r="48">
       <c r="A48" s="6" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
@@ -3156,17 +3155,17 @@
       </c>
       <c r="C48" s="6" t="inlineStr">
         <is>
-          <t>Issue / Revoke reward</t>
+          <t>Recent referrals table</t>
         </is>
       </c>
       <c r="D48" s="6" t="inlineStr">
         <is>
-          <t>Manual toggle on Referral.rewardIssued</t>
+          <t>Referee phone, rides done / 10, status (Pending/Joined/Rewarded), date</t>
         </is>
       </c>
       <c r="E48" s="6" t="inlineStr">
         <is>
-          <t>SUPER/ADMIN</t>
+          <t>same</t>
         </is>
       </c>
       <c r="F48" s="12" t="inlineStr">
@@ -3178,7 +3177,7 @@
     </row>
     <row r="49">
       <c r="A49" s="6" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
@@ -3187,12 +3186,12 @@
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>Mark joined</t>
+          <t>Issue / Revoke reward</t>
         </is>
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
-          <t>Manual toggle on refereeJoined</t>
+          <t>Manual toggle on Referral.rewardIssued</t>
         </is>
       </c>
       <c r="E49" s="6" t="inlineStr">
@@ -3209,7 +3208,7 @@
     </row>
     <row r="50">
       <c r="A50" s="6" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
@@ -3218,12 +3217,12 @@
       </c>
       <c r="C50" s="6" t="inlineStr">
         <is>
-          <t>Recompute rewards button</t>
+          <t>Mark joined</t>
         </is>
       </c>
       <c r="D50" s="6" t="inlineStr">
         <is>
-          <t>Scans all drivers, grants rewards for any who crossed 10 rides</t>
+          <t>Manual toggle on refereeJoined</t>
         </is>
       </c>
       <c r="E50" s="6" t="inlineStr">
@@ -3240,82 +3239,82 @@
     </row>
     <row r="51">
       <c r="A51" s="6" t="n">
+        <v>37</v>
+      </c>
+      <c r="B51" s="6" t="inlineStr">
+        <is>
+          <t>/referrals</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="inlineStr">
+        <is>
+          <t>Recompute rewards button</t>
+        </is>
+      </c>
+      <c r="D51" s="6" t="inlineStr">
+        <is>
+          <t>Scans all drivers, grants rewards for any who crossed 10 rides</t>
+        </is>
+      </c>
+      <c r="E51" s="6" t="inlineStr">
+        <is>
+          <t>SUPER/ADMIN</t>
+        </is>
+      </c>
+      <c r="F51" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G51" s="6" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="n">
         <v>38</v>
       </c>
-      <c r="B51" s="6" t="inlineStr">
+      <c r="B52" s="6" t="inlineStr">
         <is>
           <t>automation</t>
         </is>
       </c>
-      <c r="C51" s="6" t="inlineStr">
+      <c r="C52" s="6" t="inlineStr">
         <is>
           <t>Auto-reward on ride complete</t>
         </is>
       </c>
-      <c r="D51" s="6" t="inlineStr">
+      <c r="D52" s="6" t="inlineStr">
         <is>
           <t>On PATCH action=COMPLETE, if driver was referred + hit 10 rides, extend referrer subscriptionUntil by 7 days</t>
         </is>
       </c>
-      <c r="E51" s="6" t="inlineStr">
+      <c r="E52" s="6" t="inlineStr">
         <is>
           <t>system</t>
         </is>
       </c>
-      <c r="F51" s="12" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="G51" s="6" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="13" t="inlineStr">
+      <c r="F52" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G52" s="6" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="13" t="inlineStr">
         <is>
           <t>REPORTS</t>
         </is>
       </c>
-      <c r="B52" s="14" t="n"/>
-      <c r="C52" s="14" t="n"/>
-      <c r="D52" s="14" t="n"/>
-      <c r="E52" s="14" t="n"/>
-      <c r="F52" s="14" t="n"/>
-      <c r="G52" s="15" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="6" t="n">
-        <v>39</v>
-      </c>
-      <c r="B53" s="6" t="inlineStr">
-        <is>
-          <t>/reports</t>
-        </is>
-      </c>
-      <c r="C53" s="6" t="inlineStr">
-        <is>
-          <t>Range pills</t>
-        </is>
-      </c>
-      <c r="D53" s="6" t="inlineStr">
-        <is>
-          <t>Last 7 / 14 / 30 / 90 days</t>
-        </is>
-      </c>
-      <c r="E53" s="6" t="inlineStr">
-        <is>
-          <t>SUPER/ADMIN/CITY/SUPP/VIEW</t>
-        </is>
-      </c>
-      <c r="F53" s="12" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="G53" s="6" t="inlineStr"/>
+      <c r="B53" s="14" t="n"/>
+      <c r="C53" s="14" t="n"/>
+      <c r="D53" s="14" t="n"/>
+      <c r="E53" s="14" t="n"/>
+      <c r="F53" s="14" t="n"/>
+      <c r="G53" s="15" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="6" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B54" s="6" t="inlineStr">
         <is>
@@ -3324,17 +3323,17 @@
       </c>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>Stat cards</t>
+          <t>Range pills</t>
         </is>
       </c>
       <c r="D54" s="6" t="inlineStr">
         <is>
-          <t>Rides, revenue, completion %, active drivers</t>
+          <t>Last 7 / 14 / 30 / 90 days</t>
         </is>
       </c>
       <c r="E54" s="6" t="inlineStr">
         <is>
-          <t>same</t>
+          <t>SUPER/ADMIN/CITY/SUPP/VIEW</t>
         </is>
       </c>
       <c r="F54" s="12" t="inlineStr">
@@ -3346,7 +3345,7 @@
     </row>
     <row r="55">
       <c r="A55" s="6" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B55" s="6" t="inlineStr">
         <is>
@@ -3355,12 +3354,12 @@
       </c>
       <c r="C55" s="6" t="inlineStr">
         <is>
-          <t>Charts</t>
+          <t>Stat cards</t>
         </is>
       </c>
       <c r="D55" s="6" t="inlineStr">
         <is>
-          <t>Rides-per-day bar, revenue line, booking-channel donut</t>
+          <t>Rides, revenue, completion %, active drivers</t>
         </is>
       </c>
       <c r="E55" s="6" t="inlineStr">
@@ -3373,15 +3372,11 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G55" s="6" t="inlineStr">
-        <is>
-          <t>Chart.js</t>
-        </is>
-      </c>
+      <c r="G55" s="6" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="6" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B56" s="6" t="inlineStr">
         <is>
@@ -3390,12 +3385,12 @@
       </c>
       <c r="C56" s="6" t="inlineStr">
         <is>
-          <t>By-city breakdown</t>
+          <t>Charts</t>
         </is>
       </c>
       <c r="D56" s="6" t="inlineStr">
         <is>
-          <t>Rides, completion %, revenue per city</t>
+          <t>Rides-per-day bar, revenue line, booking-channel donut</t>
         </is>
       </c>
       <c r="E56" s="6" t="inlineStr">
@@ -3408,11 +3403,15 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G56" s="6" t="inlineStr"/>
+      <c r="G56" s="6" t="inlineStr">
+        <is>
+          <t>Chart.js</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="6" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B57" s="6" t="inlineStr">
         <is>
@@ -3421,12 +3420,12 @@
       </c>
       <c r="C57" s="6" t="inlineStr">
         <is>
-          <t>Top drivers table</t>
+          <t>By-city breakdown</t>
         </is>
       </c>
       <c r="D57" s="6" t="inlineStr">
         <is>
-          <t>Top 10 by rides + revenue</t>
+          <t>Rides, completion %, revenue per city</t>
         </is>
       </c>
       <c r="E57" s="6" t="inlineStr">
@@ -3443,86 +3442,86 @@
     </row>
     <row r="58">
       <c r="A58" s="6" t="n">
+        <v>43</v>
+      </c>
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>/reports</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="inlineStr">
+        <is>
+          <t>Top drivers table</t>
+        </is>
+      </c>
+      <c r="D58" s="6" t="inlineStr">
+        <is>
+          <t>Top 10 by rides + revenue</t>
+        </is>
+      </c>
+      <c r="E58" s="6" t="inlineStr">
+        <is>
+          <t>same</t>
+        </is>
+      </c>
+      <c r="F58" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G58" s="6" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="n">
         <v>44</v>
       </c>
-      <c r="B58" s="6" t="inlineStr">
+      <c r="B59" s="6" t="inlineStr">
         <is>
           <t>/reports</t>
         </is>
       </c>
-      <c r="C58" s="6" t="inlineStr">
+      <c r="C59" s="6" t="inlineStr">
         <is>
           <t>CSV export</t>
         </is>
       </c>
-      <c r="D58" s="6" t="inlineStr">
+      <c r="D59" s="6" t="inlineStr">
         <is>
           <t>GET /api/reports/export?days=N → rides-Nd-YYYY-MM-DD.csv</t>
         </is>
       </c>
-      <c r="E58" s="6" t="inlineStr">
+      <c r="E59" s="6" t="inlineStr">
         <is>
           <t>same</t>
         </is>
       </c>
-      <c r="F58" s="12" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="G58" s="6" t="inlineStr">
+      <c r="F59" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G59" s="6" t="inlineStr">
         <is>
           <t>City-filtered for CITY_ADMIN</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="13" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="13" t="inlineStr">
         <is>
           <t>KIRANA PARTNERS (admin side)</t>
         </is>
       </c>
-      <c r="B59" s="14" t="n"/>
-      <c r="C59" s="14" t="n"/>
-      <c r="D59" s="14" t="n"/>
-      <c r="E59" s="14" t="n"/>
-      <c r="F59" s="14" t="n"/>
-      <c r="G59" s="15" t="n"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="6" t="n">
-        <v>45</v>
-      </c>
-      <c r="B60" s="6" t="inlineStr">
-        <is>
-          <t>/partners</t>
-        </is>
-      </c>
-      <c r="C60" s="6" t="inlineStr">
-        <is>
-          <t>Partner list with status filter</t>
-        </is>
-      </c>
-      <c r="D60" s="6" t="inlineStr">
-        <is>
-          <t>Shop, owner, phone, city, commission %, bookings count, status + review note</t>
-        </is>
-      </c>
-      <c r="E60" s="6" t="inlineStr">
-        <is>
-          <t>SUPER/ADMIN/CITY (write) · VIEW (read)</t>
-        </is>
-      </c>
-      <c r="F60" s="12" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="G60" s="6" t="inlineStr"/>
+      <c r="B60" s="14" t="n"/>
+      <c r="C60" s="14" t="n"/>
+      <c r="D60" s="14" t="n"/>
+      <c r="E60" s="14" t="n"/>
+      <c r="F60" s="14" t="n"/>
+      <c r="G60" s="15" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="6" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
@@ -3531,17 +3530,17 @@
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>Approve / Reject / Suspend</t>
+          <t>Partner list with status filter</t>
         </is>
       </c>
       <c r="D61" s="6" t="inlineStr">
         <is>
-          <t>PATCH status + optional reviewNote</t>
+          <t>Shop, owner, phone, city, commission %, bookings count, status + review note</t>
         </is>
       </c>
       <c r="E61" s="6" t="inlineStr">
         <is>
-          <t>SUPER/ADMIN/CITY</t>
+          <t>SUPER/ADMIN/CITY (write) · VIEW (read)</t>
         </is>
       </c>
       <c r="F61" s="12" t="inlineStr">
@@ -3553,211 +3552,213 @@
     </row>
     <row r="62">
       <c r="A62" s="6" t="n">
+        <v>46</v>
+      </c>
+      <c r="B62" s="6" t="inlineStr">
+        <is>
+          <t>/partners</t>
+        </is>
+      </c>
+      <c r="C62" s="6" t="inlineStr">
+        <is>
+          <t>Approve / Reject / Suspend</t>
+        </is>
+      </c>
+      <c r="D62" s="6" t="inlineStr">
+        <is>
+          <t>PATCH status + optional reviewNote</t>
+        </is>
+      </c>
+      <c r="E62" s="6" t="inlineStr">
+        <is>
+          <t>SUPER/ADMIN/CITY</t>
+        </is>
+      </c>
+      <c r="F62" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G62" s="6" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="n">
         <v>47</v>
       </c>
-      <c r="B62" s="6" t="inlineStr">
+      <c r="B63" s="6" t="inlineStr">
         <is>
           <t>/partners</t>
         </is>
       </c>
-      <c r="C62" s="6" t="inlineStr">
+      <c r="C63" s="6" t="inlineStr">
         <is>
           <t>Commission % editor</t>
         </is>
       </c>
-      <c r="D62" s="6" t="inlineStr">
+      <c r="D63" s="6" t="inlineStr">
         <is>
           <t>Per-partner override (default 10%)</t>
         </is>
       </c>
-      <c r="E62" s="6" t="inlineStr">
+      <c r="E63" s="6" t="inlineStr">
         <is>
           <t>same</t>
         </is>
       </c>
-      <c r="F62" s="12" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="G62" s="6" t="inlineStr"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="13" t="inlineStr">
+      <c r="F63" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G63" s="6" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="13" t="inlineStr">
+        <is>
+          <t>SUBSCRIPTIONS</t>
+        </is>
+      </c>
+      <c r="B64" s="14" t="n"/>
+      <c r="C64" s="14" t="n"/>
+      <c r="D64" s="14" t="n"/>
+      <c r="E64" s="14" t="n"/>
+      <c r="F64" s="14" t="n"/>
+      <c r="G64" s="15" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B65" s="6" t="inlineStr">
+        <is>
+          <t>/subscriptions</t>
+        </is>
+      </c>
+      <c r="C65" s="6" t="inlineStr">
+        <is>
+          <t>Subscription list + stats</t>
+        </is>
+      </c>
+      <c r="D65" s="6" t="inlineStr">
+        <is>
+          <t>All driver plans with active/expired/revoked status; active/total/revenue cards</t>
+        </is>
+      </c>
+      <c r="E65" s="6" t="inlineStr">
+        <is>
+          <t>SUPER/ADMIN (write) · VIEW (read)</t>
+        </is>
+      </c>
+      <c r="F65" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G65" s="6" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B66" s="6" t="inlineStr">
+        <is>
+          <t>/subscriptions</t>
+        </is>
+      </c>
+      <c r="C66" s="6" t="inlineStr">
+        <is>
+          <t>Grant subscription</t>
+        </is>
+      </c>
+      <c r="D66" s="6" t="inlineStr">
+        <is>
+          <t>Pick approved driver + plan (DAILY/WEEKLY/MONTHLY) + amount; stacks on existing expiry</t>
+        </is>
+      </c>
+      <c r="E66" s="6" t="inlineStr">
+        <is>
+          <t>SUPER/ADMIN</t>
+        </is>
+      </c>
+      <c r="F66" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G66" s="6" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B67" s="6" t="inlineStr">
+        <is>
+          <t>/subscriptions</t>
+        </is>
+      </c>
+      <c r="C67" s="6" t="inlineStr">
+        <is>
+          <t>Revoke / Reinstate</t>
+        </is>
+      </c>
+      <c r="D67" s="6" t="inlineStr">
+        <is>
+          <t>PATCH active flag; rolls back driver.subscriptionUntil if all plans inactive</t>
+        </is>
+      </c>
+      <c r="E67" s="6" t="inlineStr">
+        <is>
+          <t>SUPER/ADMIN</t>
+        </is>
+      </c>
+      <c r="F67" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G67" s="6" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="13" t="inlineStr">
         <is>
           <t>ADMIN USER MGMT</t>
         </is>
       </c>
-      <c r="B63" s="14" t="n"/>
-      <c r="C63" s="14" t="n"/>
-      <c r="D63" s="14" t="n"/>
-      <c r="E63" s="14" t="n"/>
-      <c r="F63" s="14" t="n"/>
-      <c r="G63" s="15" t="n"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="6" t="n">
-        <v>48</v>
-      </c>
-      <c r="B64" s="6" t="inlineStr">
-        <is>
-          <t>/admins</t>
-        </is>
-      </c>
-      <c r="C64" s="6" t="inlineStr">
-        <is>
-          <t>Create admin form</t>
-        </is>
-      </c>
-      <c r="D64" s="6" t="inlineStr">
-        <is>
-          <t>Email, name, password (8+), role, city picker (if CITY_ADMIN)</t>
-        </is>
-      </c>
-      <c r="E64" s="6" t="inlineStr">
-        <is>
-          <t>Super Admin only</t>
-        </is>
-      </c>
-      <c r="F64" s="12" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="G64" s="6" t="inlineStr"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="6" t="n">
-        <v>49</v>
-      </c>
-      <c r="B65" s="6" t="inlineStr">
-        <is>
-          <t>/admins</t>
-        </is>
-      </c>
-      <c r="C65" s="6" t="inlineStr">
-        <is>
-          <t>Admin list</t>
-        </is>
-      </c>
-      <c r="D65" s="6" t="inlineStr">
-        <is>
-          <t>Name, email, role badge, city, active/disabled, joined</t>
-        </is>
-      </c>
-      <c r="E65" s="6" t="inlineStr">
-        <is>
-          <t>Super Admin only to see controls</t>
-        </is>
-      </c>
-      <c r="F65" s="12" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="G65" s="6" t="inlineStr">
-        <is>
-          <t>Non-super sees list read-only</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="6" t="n">
-        <v>50</v>
-      </c>
-      <c r="B66" s="6" t="inlineStr">
-        <is>
-          <t>/admins</t>
-        </is>
-      </c>
-      <c r="C66" s="6" t="inlineStr">
-        <is>
-          <t>Enable / Disable / Delete</t>
-        </is>
-      </c>
-      <c r="D66" s="6" t="inlineStr">
-        <is>
-          <t>Self-delete + self-deactivate blocked</t>
-        </is>
-      </c>
-      <c r="E66" s="6" t="inlineStr">
-        <is>
-          <t>Super Admin only</t>
-        </is>
-      </c>
-      <c r="F66" s="12" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="G66" s="6" t="inlineStr"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="13" t="inlineStr">
-        <is>
-          <t>CROSS-CUTTING</t>
-        </is>
-      </c>
-      <c r="B67" s="14" t="n"/>
-      <c r="C67" s="14" t="n"/>
-      <c r="D67" s="14" t="n"/>
-      <c r="E67" s="14" t="n"/>
-      <c r="F67" s="14" t="n"/>
-      <c r="G67" s="15" t="n"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="6" t="n">
-        <v>51</v>
-      </c>
-      <c r="B68" s="6" t="inlineStr">
-        <is>
-          <t>sidebar</t>
-        </is>
-      </c>
-      <c r="C68" s="6" t="inlineStr">
-        <is>
-          <t>Role-filtered nav</t>
-        </is>
-      </c>
-      <c r="D68" s="6" t="inlineStr">
-        <is>
-          <t>Hide pages user can't access; role label under logo</t>
-        </is>
-      </c>
-      <c r="E68" s="6" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="F68" s="12" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="G68" s="6" t="inlineStr"/>
+      <c r="B68" s="14" t="n"/>
+      <c r="C68" s="14" t="n"/>
+      <c r="D68" s="14" t="n"/>
+      <c r="E68" s="14" t="n"/>
+      <c r="F68" s="14" t="n"/>
+      <c r="G68" s="15" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="6" t="n">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>layout</t>
+          <t>/admins</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
-          <t>Session enforcement</t>
+          <t>Create admin form</t>
         </is>
       </c>
       <c r="D69" s="6" t="inlineStr">
         <is>
-          <t>requireAccess(surface) on every page; redirects unauthorized to /</t>
+          <t>Email, name, password (8+), role, city picker (if CITY_ADMIN)</t>
         </is>
       </c>
       <c r="E69" s="6" t="inlineStr">
         <is>
-          <t>all</t>
+          <t>Super Admin only</t>
         </is>
       </c>
       <c r="F69" s="12" t="inlineStr">
@@ -3769,26 +3770,26 @@
     </row>
     <row r="70">
       <c r="A70" s="6" t="n">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>API</t>
+          <t>/admins</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
         <is>
-          <t>requireWrite + cityMismatch</t>
+          <t>Admin list</t>
         </is>
       </c>
       <c r="D70" s="6" t="inlineStr">
         <is>
-          <t>Centralized guards on every API mutation</t>
+          <t>Name, email, role badge, city, active/disabled, joined</t>
         </is>
       </c>
       <c r="E70" s="6" t="inlineStr">
         <is>
-          <t>all</t>
+          <t>Super Admin only to see controls</t>
         </is>
       </c>
       <c r="F70" s="12" t="inlineStr">
@@ -3796,165 +3797,307 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G70" s="6" t="inlineStr"/>
+      <c r="G70" s="6" t="inlineStr">
+        <is>
+          <t>Non-super sees list read-only</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="6" t="n">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>global</t>
+          <t>/admins</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
         <is>
-          <t>i18n Hindi + English toggle</t>
+          <t>Enable / Disable / Delete</t>
         </is>
       </c>
       <c r="D71" s="6" t="inlineStr">
         <is>
-          <t>next-intl across all admin strings</t>
+          <t>Self-delete + self-deactivate blocked</t>
         </is>
       </c>
       <c r="E71" s="6" t="inlineStr">
         <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="F71" s="16" t="inlineStr">
-        <is>
-          <t>TODO</t>
-        </is>
-      </c>
-      <c r="G71" s="6" t="inlineStr">
-        <is>
-          <t>Tracker #20, Low priority</t>
-        </is>
-      </c>
+          <t>Super Admin only</t>
+        </is>
+      </c>
+      <c r="F71" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G71" s="6" t="inlineStr"/>
     </row>
     <row r="72">
-      <c r="A72" s="6" t="n">
-        <v>55</v>
-      </c>
-      <c r="B72" s="6" t="inlineStr">
-        <is>
-          <t>global</t>
-        </is>
-      </c>
-      <c r="C72" s="6" t="inlineStr">
-        <is>
-          <t>Audit log / compliance module</t>
-        </is>
-      </c>
-      <c r="D72" s="6" t="inlineStr">
-        <is>
-          <t>Track who changed what, when</t>
-        </is>
-      </c>
-      <c r="E72" s="6" t="inlineStr">
-        <is>
-          <t>SUPER/ADMIN</t>
-        </is>
-      </c>
-      <c r="F72" s="16" t="inlineStr">
-        <is>
-          <t>TODO</t>
-        </is>
-      </c>
-      <c r="G72" s="6" t="inlineStr">
-        <is>
-          <t>Post-MVP per SOW</t>
-        </is>
-      </c>
+      <c r="A72" s="13" t="inlineStr">
+        <is>
+          <t>CROSS-CUTTING</t>
+        </is>
+      </c>
+      <c r="B72" s="14" t="n"/>
+      <c r="C72" s="14" t="n"/>
+      <c r="D72" s="14" t="n"/>
+      <c r="E72" s="14" t="n"/>
+      <c r="F72" s="14" t="n"/>
+      <c r="G72" s="15" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="6" t="n">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>global</t>
+          <t>sidebar</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
         <is>
-          <t>Enterprise admin console</t>
+          <t>Role-filtered nav</t>
         </is>
       </c>
       <c r="D73" s="6" t="inlineStr">
         <is>
-          <t>Corporate/fleet accounts</t>
+          <t>Hide pages user can't access; role label under logo</t>
         </is>
       </c>
       <c r="E73" s="6" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F73" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G73" s="6" t="inlineStr">
-        <is>
-          <t>Post-MVP</t>
-        </is>
-      </c>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="F73" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G73" s="6" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="6" t="n">
+        <v>52</v>
+      </c>
+      <c r="B74" s="6" t="inlineStr">
+        <is>
+          <t>layout</t>
+        </is>
+      </c>
+      <c r="C74" s="6" t="inlineStr">
+        <is>
+          <t>Session enforcement</t>
+        </is>
+      </c>
+      <c r="D74" s="6" t="inlineStr">
+        <is>
+          <t>requireAccess(surface) on every page; redirects unauthorized to /</t>
+        </is>
+      </c>
+      <c r="E74" s="6" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="F74" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G74" s="6" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="6" t="n">
+        <v>53</v>
+      </c>
+      <c r="B75" s="6" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="C75" s="6" t="inlineStr">
+        <is>
+          <t>requireWrite + cityMismatch</t>
+        </is>
+      </c>
+      <c r="D75" s="6" t="inlineStr">
+        <is>
+          <t>Centralized guards on every API mutation</t>
+        </is>
+      </c>
+      <c r="E75" s="6" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="F75" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G75" s="6" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="6" t="n">
+        <v>54</v>
+      </c>
+      <c r="B76" s="6" t="inlineStr">
+        <is>
+          <t>global</t>
+        </is>
+      </c>
+      <c r="C76" s="6" t="inlineStr">
+        <is>
+          <t>i18n Hindi + English toggle</t>
+        </is>
+      </c>
+      <c r="D76" s="6" t="inlineStr">
+        <is>
+          <t>next-intl across all admin strings</t>
+        </is>
+      </c>
+      <c r="E76" s="6" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="F76" s="16" t="inlineStr">
+        <is>
+          <t>TODO</t>
+        </is>
+      </c>
+      <c r="G76" s="6" t="inlineStr">
+        <is>
+          <t>Tracker #20, Low priority</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="6" t="n">
+        <v>55</v>
+      </c>
+      <c r="B77" s="6" t="inlineStr">
+        <is>
+          <t>global</t>
+        </is>
+      </c>
+      <c r="C77" s="6" t="inlineStr">
+        <is>
+          <t>Audit log / compliance module</t>
+        </is>
+      </c>
+      <c r="D77" s="6" t="inlineStr">
+        <is>
+          <t>Track who changed what, when</t>
+        </is>
+      </c>
+      <c r="E77" s="6" t="inlineStr">
+        <is>
+          <t>SUPER/ADMIN</t>
+        </is>
+      </c>
+      <c r="F77" s="16" t="inlineStr">
+        <is>
+          <t>TODO</t>
+        </is>
+      </c>
+      <c r="G77" s="6" t="inlineStr">
+        <is>
+          <t>Post-MVP per SOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="6" t="n">
+        <v>56</v>
+      </c>
+      <c r="B78" s="6" t="inlineStr">
+        <is>
+          <t>global</t>
+        </is>
+      </c>
+      <c r="C78" s="6" t="inlineStr">
+        <is>
+          <t>Enterprise admin console</t>
+        </is>
+      </c>
+      <c r="D78" s="6" t="inlineStr">
+        <is>
+          <t>Corporate/fleet accounts</t>
+        </is>
+      </c>
+      <c r="E78" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F78" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G78" s="6" t="inlineStr">
+        <is>
+          <t>Post-MVP</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="6" t="n">
         <v>57</v>
       </c>
-      <c r="B74" s="6" t="inlineStr">
+      <c r="B79" s="6" t="inlineStr">
         <is>
           <t>global</t>
         </is>
       </c>
-      <c r="C74" s="6" t="inlineStr">
+      <c r="C79" s="6" t="inlineStr">
         <is>
           <t>Socket.io realtime rides</t>
         </is>
       </c>
-      <c r="D74" s="6" t="inlineStr">
+      <c r="D79" s="6" t="inlineStr">
         <is>
           <t>Replace polling with live push</t>
         </is>
       </c>
-      <c r="E74" s="6" t="inlineStr">
+      <c r="E79" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F74" s="16" t="inlineStr">
+      <c r="F79" s="16" t="inlineStr">
         <is>
           <t>TODO</t>
         </is>
       </c>
-      <c r="G74" s="6" t="inlineStr">
+      <c r="G79" s="6" t="inlineStr">
         <is>
           <t>Backend dependency</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="15">
-    <mergeCell ref="A36:G36"/>
-    <mergeCell ref="A44:G44"/>
+  <mergeCells count="16">
+    <mergeCell ref="A32:G32"/>
     <mergeCell ref="A17:G17"/>
     <mergeCell ref="A9:G9"/>
-    <mergeCell ref="A40:G40"/>
-    <mergeCell ref="A31:G31"/>
-    <mergeCell ref="A67:G67"/>
+    <mergeCell ref="A45:G45"/>
     <mergeCell ref="A21:G21"/>
-    <mergeCell ref="A34:G34"/>
+    <mergeCell ref="A53:G53"/>
+    <mergeCell ref="A35:G35"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A72:G72"/>
     <mergeCell ref="A29:G29"/>
-    <mergeCell ref="A52:G52"/>
-    <mergeCell ref="A59:G59"/>
-    <mergeCell ref="A63:G63"/>
+    <mergeCell ref="A64:G64"/>
+    <mergeCell ref="A60:G60"/>
+    <mergeCell ref="A41:G41"/>
+    <mergeCell ref="A68:G68"/>
     <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A37:G37"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3966,7 +4109,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -4470,12 +4613,12 @@
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>Map-based pickup picker</t>
+          <t>Map-based pickup/drop picker</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>Click map / search to set pickup</t>
+          <t>Leaflet + OSM Nominatim; click map or search address to set pickup and drop</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
@@ -4483,16 +4626,12 @@
           <t>same</t>
         </is>
       </c>
-      <c r="F18" s="16" t="inlineStr">
-        <is>
-          <t>TODO</t>
-        </is>
-      </c>
-      <c r="G18" s="6" t="inlineStr">
-        <is>
-          <t>Requires Google Places or OSM Nominatim</t>
-        </is>
-      </c>
+      <c r="F18" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="6" t="n">
@@ -4829,12 +4968,12 @@
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>KYC document upload</t>
+          <t>KYC document upload + status</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>Shop license, aadhaar, etc.</t>
+          <t>Pick type + file, upload to /api/kirana/documents; shows per-doc PENDING/APPROVED/REJECTED badge</t>
         </is>
       </c>
       <c r="E29" s="6" t="inlineStr">
@@ -4842,16 +4981,12 @@
           <t>same</t>
         </is>
       </c>
-      <c r="F29" s="16" t="inlineStr">
-        <is>
-          <t>TODO</t>
-        </is>
-      </c>
-      <c r="G29" s="6" t="inlineStr">
-        <is>
-          <t>PartnerDocument model exists, no upload UI</t>
-        </is>
-      </c>
+      <c r="F29" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="13" t="inlineStr">
@@ -4931,7 +5066,7 @@
     <row r="33">
       <c r="A33" s="13" t="inlineStr">
         <is>
-          <t>CROSS-CUTTING</t>
+          <t>PWA SHELL</t>
         </is>
       </c>
       <c r="B33" s="14" t="n"/>
@@ -4942,206 +5077,366 @@
       <c r="G33" s="15" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="6" t="n">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>manifest</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>Web App Manifest</t>
+        </is>
+      </c>
+      <c r="D34" s="6" t="inlineStr">
+        <is>
+          <t>public/manifest.webmanifest scoped to /k/ with name/icons/theme/start_url</t>
+        </is>
+      </c>
+      <c r="E34" s="6" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F34" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G34" s="6" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>icons</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>App icons + apple-touch</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="inlineStr">
+        <is>
+          <t>192/512 PNG + maskable 512 + 180 apple-touch, brand orange 'GG' monogram</t>
+        </is>
+      </c>
+      <c r="E35" s="6" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F35" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G35" s="6" t="inlineStr">
+        <is>
+          <t>Generated via scripts/build-pwa-icons.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>service-worker</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>Service worker (/sw.js, scope /k/)</t>
+        </is>
+      </c>
+      <c r="D36" s="6" t="inlineStr">
+        <is>
+          <t>Cache-first static, network-first kirana APIs, offline fallback to /offline.html</t>
+        </is>
+      </c>
+      <c r="E36" s="6" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F36" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G36" s="6" t="inlineStr">
+        <is>
+          <t>Service-Worker-Allowed header set in next.config.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>install</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>Install prompt component</t>
+        </is>
+      </c>
+      <c r="D37" s="6" t="inlineStr">
+        <is>
+          <t>Captures beforeinstallprompt, shows 'Add to home screen' banner with dismiss persistence</t>
+        </is>
+      </c>
+      <c r="E37" s="6" t="inlineStr">
+        <is>
+          <t>Approved partner</t>
+        </is>
+      </c>
+      <c r="F37" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G37" s="6" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>push</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>Push notifications</t>
+        </is>
+      </c>
+      <c r="D38" s="6" t="inlineStr">
+        <is>
+          <t>Driver matched / arrived / completed alerts</t>
+        </is>
+      </c>
+      <c r="E38" s="6" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="F38" s="16" t="inlineStr">
+        <is>
+          <t>TODO</t>
+        </is>
+      </c>
+      <c r="G38" s="6" t="inlineStr">
+        <is>
+          <t>SW ready; needs VAPID + backend trigger</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="13" t="inlineStr">
+        <is>
+          <t>CROSS-CUTTING</t>
+        </is>
+      </c>
+      <c r="B39" s="14" t="n"/>
+      <c r="C39" s="14" t="n"/>
+      <c r="D39" s="14" t="n"/>
+      <c r="E39" s="14" t="n"/>
+      <c r="F39" s="14" t="n"/>
+      <c r="G39" s="15" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="n">
         <v>24</v>
       </c>
-      <c r="B34" s="6" t="inlineStr">
+      <c r="B40" s="6" t="inlineStr">
         <is>
           <t>OTP</t>
         </is>
       </c>
-      <c r="C34" s="6" t="inlineStr">
+      <c r="C40" s="6" t="inlineStr">
         <is>
           <t>6-digit, 5-min TTL</t>
         </is>
       </c>
-      <c r="D34" s="6" t="inlineStr">
+      <c r="D40" s="6" t="inlineStr">
         <is>
           <t>OtpRequest table; single-use (usedAt timestamp)</t>
         </is>
       </c>
-      <c r="E34" s="6" t="inlineStr">
+      <c r="E40" s="6" t="inlineStr">
         <is>
           <t>system</t>
         </is>
       </c>
-      <c r="F34" s="12" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="G34" s="6" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="6" t="n">
+      <c r="F40" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G40" s="6" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="n">
         <v>25</v>
       </c>
-      <c r="B35" s="6" t="inlineStr">
+      <c r="B41" s="6" t="inlineStr">
         <is>
           <t>OTP</t>
         </is>
       </c>
-      <c r="C35" s="6" t="inlineStr">
+      <c r="C41" s="6" t="inlineStr">
         <is>
           <t>MSG91 send</t>
         </is>
       </c>
-      <c r="D35" s="6" t="inlineStr">
+      <c r="D41" s="6" t="inlineStr">
         <is>
           <t>Actually send the code via SMS</t>
         </is>
       </c>
-      <c r="E35" s="6" t="inlineStr">
+      <c r="E41" s="6" t="inlineStr">
         <is>
           <t>system</t>
         </is>
       </c>
-      <c r="F35" s="16" t="inlineStr">
+      <c r="F41" s="16" t="inlineStr">
         <is>
           <t>TODO</t>
         </is>
       </c>
-      <c r="G35" s="6" t="inlineStr">
+      <c r="G41" s="6" t="inlineStr">
         <is>
           <t>Stubbed; returns devCode in dev</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="6" t="n">
+    <row r="42">
+      <c r="A42" s="6" t="n">
         <v>26</v>
       </c>
-      <c r="B36" s="6" t="inlineStr">
+      <c r="B42" s="6" t="inlineStr">
         <is>
           <t>fare</t>
         </is>
       </c>
-      <c r="C36" s="6" t="inlineStr">
+      <c r="C42" s="6" t="inlineStr">
         <is>
           <t>Haversine + concession</t>
         </is>
       </c>
-      <c r="D36" s="6" t="inlineStr">
+      <c r="D42" s="6" t="inlineStr">
         <is>
           <t>src/lib/fare.ts shared with future rider/driver apps</t>
         </is>
       </c>
-      <c r="E36" s="6" t="inlineStr">
+      <c r="E42" s="6" t="inlineStr">
         <is>
           <t>system</t>
         </is>
       </c>
-      <c r="F36" s="12" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="G36" s="6" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="6" t="n">
+      <c r="F42" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G42" s="6" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="n">
         <v>27</v>
       </c>
-      <c r="B37" s="6" t="inlineStr">
+      <c r="B43" s="6" t="inlineStr">
         <is>
           <t>commission</t>
         </is>
       </c>
-      <c r="C37" s="6" t="inlineStr">
+      <c r="C43" s="6" t="inlineStr">
         <is>
           <t>Payout / settlement</t>
         </is>
       </c>
-      <c r="D37" s="6" t="inlineStr">
+      <c r="D43" s="6" t="inlineStr">
         <is>
           <t>Actually paying partners their earned commission</t>
         </is>
       </c>
-      <c r="E37" s="6" t="inlineStr">
+      <c r="E43" s="6" t="inlineStr">
         <is>
           <t>system</t>
         </is>
       </c>
-      <c r="F37" s="16" t="inlineStr">
+      <c r="F43" s="16" t="inlineStr">
         <is>
           <t>TODO</t>
         </is>
       </c>
-      <c r="G37" s="6" t="inlineStr">
+      <c r="G43" s="6" t="inlineStr">
         <is>
           <t>Tracks earned; no payout flow</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="6" t="n">
-        <v>28</v>
-      </c>
-      <c r="B38" s="6" t="inlineStr">
-        <is>
-          <t>push</t>
-        </is>
-      </c>
-      <c r="C38" s="6" t="inlineStr">
-        <is>
-          <t>Booking status notifications</t>
-        </is>
-      </c>
-      <c r="D38" s="6" t="inlineStr">
-        <is>
-          <t>Driver matched / arrived / completed alerts</t>
-        </is>
-      </c>
-      <c r="E38" s="6" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="B44" s="6" t="inlineStr">
+        <is>
+          <t>i18n</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="inlineStr">
+        <is>
+          <t>Hindi + English toggle</t>
+        </is>
+      </c>
+      <c r="D44" s="6" t="inlineStr">
+        <is>
+          <t>react-i18next across all kirana strings</t>
+        </is>
+      </c>
+      <c r="E44" s="6" t="inlineStr">
         <is>
           <t>system</t>
         </is>
       </c>
-      <c r="F38" s="16" t="inlineStr">
+      <c r="F44" s="16" t="inlineStr">
         <is>
           <t>TODO</t>
         </is>
       </c>
-      <c r="G38" s="6" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="6" t="n">
-        <v>29</v>
-      </c>
-      <c r="B39" s="6" t="inlineStr">
-        <is>
-          <t>i18n</t>
-        </is>
-      </c>
-      <c r="C39" s="6" t="inlineStr">
-        <is>
-          <t>Hindi + English toggle</t>
-        </is>
-      </c>
-      <c r="D39" s="6" t="inlineStr">
-        <is>
-          <t>react-i18next across all kirana strings</t>
-        </is>
-      </c>
-      <c r="E39" s="6" t="inlineStr">
-        <is>
-          <t>system</t>
-        </is>
-      </c>
-      <c r="F39" s="16" t="inlineStr">
-        <is>
-          <t>TODO</t>
-        </is>
-      </c>
-      <c r="G39" s="6" t="inlineStr">
+      <c r="G44" s="6" t="inlineStr">
         <is>
           <t>Low priority</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="A8:G8"/>
+    <mergeCell ref="A39:G39"/>
     <mergeCell ref="A30:G30"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A33:G33"/>
@@ -5157,7 +5452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5413,7 +5708,7 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>PATCH</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -5423,12 +5718,12 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Approve/reject driver doc + review note</t>
+          <t>Fetch single driver document</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>documents:write + city scope</t>
+          <t>documents:read + city scope</t>
         </is>
       </c>
       <c r="E10" s="12" t="inlineStr">
@@ -5445,17 +5740,17 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>/api/rides/[id]</t>
+          <t>/api/drivers/[id]/documents/[docId]</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Cancel / Complete / Reassign driver</t>
+          <t>Approve/reject driver doc + review note</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>rides:write + city scope</t>
+          <t>documents:write + city scope</t>
         </is>
       </c>
       <c r="E11" s="12" t="inlineStr">
@@ -5467,22 +5762,22 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>/api/rides/[id]/token</t>
+          <t>/api/drivers/[id]/documents/[docId]</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Generate or fetch public tracking token</t>
+          <t>Delete driver doc + file</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>rides:write + city scope</t>
+          <t>documents:write + city scope</t>
         </is>
       </c>
       <c r="E12" s="12" t="inlineStr">
@@ -5499,17 +5794,17 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>/api/coupons</t>
+          <t>/api/uploads/driver-doc</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Create coupon</t>
+          <t>Upload driver doc file to storage</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>coupons:write</t>
+          <t>documents:write + city scope</t>
         </is>
       </c>
       <c r="E13" s="12" t="inlineStr">
@@ -5521,22 +5816,22 @@
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>PATCH</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>/api/coupons/[id]</t>
+          <t>/api/riders</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Toggle active</t>
+          <t>List riders (q/limit/offset)</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>coupons:write</t>
+          <t>riders:read</t>
         </is>
       </c>
       <c r="E14" s="12" t="inlineStr">
@@ -5548,22 +5843,22 @@
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>/api/coupons/[id]</t>
+          <t>/api/riders/[id]</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Delete coupon</t>
+          <t>Rider detail with recent rides + stats</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>coupons:write</t>
+          <t>riders:read</t>
         </is>
       </c>
       <c r="E15" s="12" t="inlineStr">
@@ -5575,22 +5870,22 @@
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>PATCH</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>/api/referrals/[id]</t>
+          <t>/api/subscriptions</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>Manual reward issue/revoke</t>
+          <t>List subscriptions (optional driverId/active filters)</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>referrals:write</t>
+          <t>subscriptions:read</t>
         </is>
       </c>
       <c r="E16" s="12" t="inlineStr">
@@ -5607,17 +5902,17 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>/api/referrals/recompute</t>
+          <t>/api/subscriptions</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>Recompute all pending referral rewards</t>
+          <t>Grant subscription (stacks on existing expiry)</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>referrals:write</t>
+          <t>subscriptions:write</t>
         </is>
       </c>
       <c r="E17" s="12" t="inlineStr">
@@ -5629,22 +5924,22 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>/api/reports/export</t>
+          <t>/api/subscriptions/[id]</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>CSV download, city-filtered</t>
+          <t>Revoke / reinstate subscription</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>reports:read</t>
+          <t>subscriptions:write</t>
         </is>
       </c>
       <c r="E18" s="12" t="inlineStr">
@@ -5656,22 +5951,22 @@
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>/api/sos</t>
+          <t>/api/rides/[id]</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Active SOS count (sidebar badge)</t>
+          <t>Cancel / Complete / Reassign driver</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>sos:read + city filter</t>
+          <t>rides:write + city scope</t>
         </is>
       </c>
       <c r="E19" s="12" t="inlineStr">
@@ -5688,17 +5983,17 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>/api/admins</t>
+          <t>/api/rides/[id]/token</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Create admin user</t>
+          <t>Generate or fetch public tracking token</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>SUPER_ADMIN</t>
+          <t>rides:write + city scope</t>
         </is>
       </c>
       <c r="E20" s="12" t="inlineStr">
@@ -5710,22 +6005,22 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>PATCH</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>/api/admins/[id]</t>
+          <t>/api/coupons</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Enable/disable, change role/city/password</t>
+          <t>Create coupon</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>SUPER_ADMIN</t>
+          <t>coupons:write</t>
         </is>
       </c>
       <c r="E21" s="12" t="inlineStr">
@@ -5737,22 +6032,22 @@
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>/api/admins/[id]</t>
+          <t>/api/coupons/[id]</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>Delete admin</t>
+          <t>Toggle active</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>SUPER_ADMIN</t>
+          <t>coupons:write</t>
         </is>
       </c>
       <c r="E22" s="12" t="inlineStr">
@@ -5764,22 +6059,22 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>PATCH</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>/api/partners/[id]</t>
+          <t>/api/coupons/[id]</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Approve/reject/suspend + commission %</t>
+          <t>Delete coupon</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>partners:write + city scope</t>
+          <t>coupons:write</t>
         </is>
       </c>
       <c r="E23" s="12" t="inlineStr">
@@ -5791,22 +6086,22 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>/api/track/[token]</t>
+          <t>/api/referrals/[id]</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>Public ride state for tracking page</t>
+          <t>Manual reward issue/revoke</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>referrals:write</t>
         </is>
       </c>
       <c r="E24" s="12" t="inlineStr">
@@ -5823,17 +6118,17 @@
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>/api/kirana/signup</t>
+          <t>/api/referrals/recompute</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>Partner application (creates PENDING)</t>
+          <t>Recompute all pending referral rewards</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>referrals:write</t>
         </is>
       </c>
       <c r="E25" s="12" t="inlineStr">
@@ -5845,22 +6140,22 @@
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>/api/kirana/otp/request</t>
+          <t>/api/reports/export</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>Generate 6-digit OTP (phone must belong to a partner)</t>
+          <t>CSV download, city-filtered</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>reports:read</t>
         </is>
       </c>
       <c r="E26" s="12" t="inlineStr">
@@ -5872,22 +6167,22 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>/api/kirana/otp/verify</t>
+          <t>/api/sos</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Verify OTP + set kirana session cookie</t>
+          <t>Active SOS count (sidebar badge)</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>sos:read + city filter</t>
         </is>
       </c>
       <c r="E27" s="12" t="inlineStr">
@@ -5904,17 +6199,17 @@
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>/api/kirana/logout</t>
+          <t>/api/admins</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>Clear kirana session</t>
+          <t>Create admin user</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>kirana session</t>
+          <t>SUPER_ADMIN</t>
         </is>
       </c>
       <c r="E28" s="12" t="inlineStr">
@@ -5926,22 +6221,22 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>PUT</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>/api/kirana/bookings</t>
+          <t>/api/admins/[id]</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>Fare estimate without creating</t>
+          <t>Enable/disable, change role/city/password</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>kirana session (any status)</t>
+          <t>SUPER_ADMIN</t>
         </is>
       </c>
       <c r="E29" s="12" t="inlineStr">
@@ -5953,25 +6248,241 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
+          <t>DELETE</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>/api/admins/[id]</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>Delete admin</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>SUPER_ADMIN</t>
+        </is>
+      </c>
+      <c r="E30" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>PATCH</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>/api/partners/[id]</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>Approve/reject/suspend + commission %</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t>partners:write + city scope</t>
+        </is>
+      </c>
+      <c r="E31" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>/api/track/[token]</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>Public ride state for tracking page</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="E32" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="B30" s="6" t="inlineStr">
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>/api/kirana/signup</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>Partner application (creates PENDING)</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="E33" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>/api/kirana/otp/request</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>Generate 6-digit OTP (phone must belong to a partner)</t>
+        </is>
+      </c>
+      <c r="D34" s="6" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="E34" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>/api/kirana/otp/verify</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>Verify OTP + set kirana session cookie</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="E35" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>/api/kirana/logout</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>Clear kirana session</t>
+        </is>
+      </c>
+      <c r="D36" s="6" t="inlineStr">
+        <is>
+          <t>kirana session</t>
+        </is>
+      </c>
+      <c r="E36" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
         <is>
           <t>/api/kirana/bookings</t>
         </is>
       </c>
-      <c r="C30" s="6" t="inlineStr">
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>Fare estimate without creating</t>
+        </is>
+      </c>
+      <c r="D37" s="6" t="inlineStr">
+        <is>
+          <t>kirana session (any status)</t>
+        </is>
+      </c>
+      <c r="E37" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>/api/kirana/bookings</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
         <is>
           <t>Create booking (REQUESTED ride with bookedByPartnerId)</t>
         </is>
       </c>
-      <c r="D30" s="6" t="inlineStr">
+      <c r="D38" s="6" t="inlineStr">
         <is>
           <t>kirana session (APPROVED only)</t>
         </is>
       </c>
-      <c r="E30" s="12" t="inlineStr">
+      <c r="E38" s="12" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -6178,12 +6689,12 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>driver detail</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>Done (no upload UI)</t>
+          <t>driver detail + upload UI</t>
+        </is>
+      </c>
+      <c r="E7" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -6556,12 +7067,12 @@
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>Referral reward extends this</t>
+          <t>/subscriptions admin + referral reward extends this</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>Schema only (no purchase UI)</t>
+          <t>Done (admin grant; no driver-side purchase UI)</t>
         </is>
       </c>
     </row>
@@ -6660,12 +7171,12 @@
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>Schema only (no UI)</t>
-        </is>
-      </c>
-      <c r="E25" s="18" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>Kirana /k/profile upload + /partners/[id] review</t>
+        </is>
+      </c>
+      <c r="E25" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -6734,7 +7245,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -7376,12 +7887,12 @@
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>Need Vercel Blob or S3</t>
+          <t>Shipped — stored under public/uploads/ in dev; production should swap to Vercel Blob / S3</t>
         </is>
       </c>
     </row>
@@ -7586,12 +8097,12 @@
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>Google Places or Nominatim</t>
+          <t>Shipped — Leaflet + Nominatim</t>
         </is>
       </c>
     </row>
@@ -7629,6 +8140,142 @@
           <t>SOW explicitly deferred to Phase 2</t>
         </is>
       </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>Driver subscription purchase UI</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>Driver PWA</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>App Dev + Backend</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>Drivers buying their own plan; admin grant exists</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>Admin /subscriptions shipped; waits on payments + Driver app</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>VAPID push notifications</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>RN/PWA + Backend</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>App Dev + Backend</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>Booking status push to kirana partners</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>PWA service worker ready; needs backend trigger + VAPID keys</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>Bookings detail + live track in Kirana PWA</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>Kirana PWA</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>Partner can't watch a ride they booked</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>Token API + public /track page already exist</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>Per-document DELETE in partner docs review</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="inlineStr">
+        <is>
+          <t>Admins can approve/reject but not remove partner docs</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>